<commit_message>
upd positions, add L_sys on nav layer
</commit_message>
<xml_diff>
--- a/assets/keys_positions.xlsx
+++ b/assets/keys_positions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://epam-my.sharepoint.com/personal/oleksii_holik_epam_com/Documents/!MyDocs/Lections/ergo-s1v1-zmk-shield-module/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9BAB8B5-5878-4489-888E-90875CF9A17F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="8_{D9BAB8B5-5878-4489-888E-90875CF9A17F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2794BB4D-0EFA-4BA1-8C62-3231B3D32D4F}"/>
   <bookViews>
-    <workbookView xWindow="45972" yWindow="5688" windowWidth="23256" windowHeight="12456" xr2:uid="{DEADC791-3ADA-4A6F-9015-8969786FFBED}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="38580" windowHeight="21060" xr2:uid="{DEADC791-3ADA-4A6F-9015-8969786FFBED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,10 +33,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -469,386 +465,266 @@
       <c r="F1" s="2">
         <v>5</v>
       </c>
-      <c r="G1" s="3">
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="2">
         <v>6</v>
       </c>
-      <c r="H1" s="3">
+      <c r="M1" s="2">
         <v>7</v>
       </c>
-      <c r="J1" s="3">
+      <c r="N1" s="2">
         <v>8</v>
       </c>
-      <c r="K1" s="3">
+      <c r="O1" s="2">
         <v>9</v>
       </c>
-      <c r="L1" s="2">
+      <c r="P1" s="2">
         <v>10</v>
       </c>
-      <c r="M1" s="2">
+      <c r="Q1" s="2">
         <v>11</v>
-      </c>
-      <c r="N1" s="2">
-        <v>12</v>
-      </c>
-      <c r="O1" s="2">
-        <v>13</v>
-      </c>
-      <c r="P1" s="2">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="2">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2">
+        <v>13</v>
+      </c>
+      <c r="C2" s="2">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2">
+        <v>15</v>
+      </c>
+      <c r="E2" s="2">
         <v>16</v>
       </c>
-      <c r="B2" s="2">
+      <c r="F2" s="2">
         <v>17</v>
       </c>
-      <c r="C2" s="2">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="2">
         <v>18</v>
       </c>
-      <c r="D2" s="2">
+      <c r="M2" s="2">
         <v>19</v>
       </c>
-      <c r="E2" s="2">
+      <c r="N2" s="2">
         <v>20</v>
       </c>
-      <c r="F2" s="2">
+      <c r="O2" s="2">
         <v>21</v>
       </c>
-      <c r="G2" s="3">
+      <c r="P2" s="2">
         <v>22</v>
       </c>
-      <c r="H2" s="3">
+      <c r="Q2" s="2">
         <v>23</v>
-      </c>
-      <c r="J2" s="3">
-        <v>24</v>
-      </c>
-      <c r="K2" s="3">
-        <v>25</v>
-      </c>
-      <c r="L2" s="2">
-        <v>26</v>
-      </c>
-      <c r="M2" s="2">
-        <v>27</v>
-      </c>
-      <c r="N2" s="2">
-        <v>28</v>
-      </c>
-      <c r="O2" s="2">
-        <v>29</v>
-      </c>
-      <c r="P2" s="2">
-        <v>30</v>
-      </c>
-      <c r="Q2" s="2">
-        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
+        <v>24</v>
+      </c>
+      <c r="B3" s="2">
+        <v>25</v>
+      </c>
+      <c r="C3" s="2">
+        <v>26</v>
+      </c>
+      <c r="D3" s="2">
+        <v>27</v>
+      </c>
+      <c r="E3" s="2">
+        <v>28</v>
+      </c>
+      <c r="F3" s="2">
+        <v>29</v>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="2">
+        <v>30</v>
+      </c>
+      <c r="M3" s="2">
+        <v>31</v>
+      </c>
+      <c r="N3" s="2">
         <v>32</v>
       </c>
-      <c r="B3" s="2">
+      <c r="O3" s="2">
         <v>33</v>
       </c>
-      <c r="C3" s="2">
+      <c r="P3" s="2">
         <v>34</v>
       </c>
-      <c r="D3" s="2">
+      <c r="Q3" s="2">
         <v>35</v>
-      </c>
-      <c r="E3" s="2">
-        <v>36</v>
-      </c>
-      <c r="F3" s="2">
-        <v>37</v>
-      </c>
-      <c r="G3" s="3">
-        <v>38</v>
-      </c>
-      <c r="H3" s="3">
-        <v>39</v>
-      </c>
-      <c r="J3" s="3">
-        <v>40</v>
-      </c>
-      <c r="K3" s="3">
-        <v>41</v>
-      </c>
-      <c r="L3" s="2">
-        <v>42</v>
-      </c>
-      <c r="M3" s="2">
-        <v>43</v>
-      </c>
-      <c r="N3" s="2">
-        <v>44</v>
-      </c>
-      <c r="O3" s="2">
-        <v>45</v>
-      </c>
-      <c r="P3" s="2">
-        <v>46</v>
-      </c>
-      <c r="Q3" s="2">
-        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="B4" s="2">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="C4" s="2">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="D4" s="2">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="E4" s="2">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="F4" s="2">
-        <v>53</v>
-      </c>
-      <c r="G4" s="3">
-        <v>54</v>
-      </c>
-      <c r="H4" s="3">
-        <v>55</v>
-      </c>
-      <c r="J4" s="3">
-        <v>56</v>
-      </c>
-      <c r="K4" s="3">
-        <v>57</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
       <c r="L4" s="2">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="M4" s="2">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="N4" s="2">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="O4" s="2">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="P4" s="2">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="Q4" s="2">
-        <v>63</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="3">
-        <v>64</v>
-      </c>
+      <c r="A5" s="3"/>
       <c r="B5" s="2">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="C5" s="2">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="D5" s="2">
-        <v>67</v>
-      </c>
-      <c r="E5" s="3">
-        <v>68</v>
-      </c>
-      <c r="F5" s="3">
-        <v>69</v>
-      </c>
-      <c r="G5" s="3">
-        <v>70</v>
-      </c>
-      <c r="H5" s="3">
-        <v>71</v>
-      </c>
-      <c r="J5" s="3">
-        <v>72</v>
-      </c>
-      <c r="K5" s="3">
-        <v>73</v>
-      </c>
-      <c r="L5" s="3">
-        <v>74</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
       <c r="M5" s="2">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="N5" s="2">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="O5" s="2">
-        <v>77</v>
-      </c>
-      <c r="P5" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q5" s="3">
-        <v>79</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
     </row>
     <row r="6" spans="1:17" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="3">
-        <v>80</v>
-      </c>
-      <c r="B6" s="3">
-        <v>81</v>
-      </c>
-      <c r="C6" s="3">
-        <v>82</v>
-      </c>
-      <c r="D6" s="3">
-        <v>83</v>
-      </c>
-      <c r="E6" s="3">
-        <v>84</v>
-      </c>
-      <c r="F6" s="3">
-        <v>85</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
       <c r="G6" s="2">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="H6" s="2">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="J6" s="2">
-        <v>88</v>
+        <v>56</v>
       </c>
       <c r="K6" s="2">
-        <v>89</v>
-      </c>
-      <c r="L6" s="3">
-        <v>90</v>
-      </c>
-      <c r="M6" s="3">
-        <v>91</v>
-      </c>
-      <c r="N6" s="3">
-        <v>92</v>
-      </c>
-      <c r="O6" s="3">
-        <v>93</v>
-      </c>
-      <c r="P6" s="3">
-        <v>94</v>
-      </c>
-      <c r="Q6" s="3">
-        <v>95</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
     </row>
     <row r="7" spans="1:17" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="3">
-        <v>96</v>
-      </c>
-      <c r="B7" s="3">
-        <v>97</v>
-      </c>
-      <c r="C7" s="3">
-        <v>98</v>
-      </c>
-      <c r="D7" s="3">
-        <v>99</v>
-      </c>
-      <c r="E7" s="3">
-        <v>100</v>
-      </c>
-      <c r="F7" s="3">
-        <v>101</v>
-      </c>
-      <c r="G7" s="3">
-        <v>102</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
       <c r="H7" s="2">
-        <v>103</v>
+        <v>58</v>
       </c>
       <c r="J7" s="2">
-        <v>104</v>
-      </c>
-      <c r="K7" s="3">
-        <v>105</v>
-      </c>
-      <c r="L7" s="3">
-        <v>106</v>
-      </c>
-      <c r="M7" s="3">
-        <v>107</v>
-      </c>
-      <c r="N7" s="3">
-        <v>108</v>
-      </c>
-      <c r="O7" s="3">
-        <v>109</v>
-      </c>
-      <c r="P7" s="3">
-        <v>110</v>
-      </c>
-      <c r="Q7" s="3">
-        <v>111</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
     </row>
     <row r="8" spans="1:17" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="3">
-        <v>112</v>
-      </c>
-      <c r="B8" s="3">
-        <v>113</v>
-      </c>
-      <c r="C8" s="3">
-        <v>114</v>
-      </c>
-      <c r="D8" s="3">
-        <v>115</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
       <c r="E8" s="2">
-        <v>116</v>
+        <v>60</v>
       </c>
       <c r="F8" s="2">
-        <v>117</v>
+        <v>61</v>
       </c>
       <c r="G8" s="2">
-        <v>118</v>
+        <v>62</v>
       </c>
       <c r="H8" s="2">
-        <v>119</v>
+        <v>63</v>
       </c>
       <c r="J8" s="2">
-        <v>120</v>
+        <v>64</v>
       </c>
       <c r="K8" s="2">
-        <v>121</v>
+        <v>65</v>
       </c>
       <c r="L8" s="2">
-        <v>122</v>
+        <v>66</v>
       </c>
       <c r="M8" s="2">
-        <v>123</v>
-      </c>
-      <c r="N8" s="3">
-        <v>124</v>
-      </c>
-      <c r="O8" s="3">
-        <v>125</v>
-      </c>
-      <c r="P8" s="3">
-        <v>126</v>
-      </c>
-      <c r="Q8" s="3">
-        <v>127</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
     </row>
     <row r="9" spans="1:17" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>

</xml_diff>